<commit_message>
ci: add main.yml workflow with 6-module 1800 test cases and master report deployment
</commit_message>
<xml_diff>
--- a/arogya_ai_flutter/automation/reports/Excel/Passed_Test_Cases.xlsx
+++ b/arogya_ai_flutter/automation/reports/Excel/Passed_Test_Cases.xlsx
@@ -3554,7 +3554,7 @@
         <v>10</v>
       </c>
       <c r="F2">
-        <v>235</v>
+        <v>740</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -3574,7 +3574,7 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>336</v>
+        <v>927</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -3594,7 +3594,7 @@
         <v>10</v>
       </c>
       <c r="F4">
-        <v>476</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -3614,7 +3614,7 @@
         <v>10</v>
       </c>
       <c r="F5">
-        <v>389</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -3634,7 +3634,7 @@
         <v>10</v>
       </c>
       <c r="F6">
-        <v>651</v>
+        <v>995</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3654,7 +3654,7 @@
         <v>10</v>
       </c>
       <c r="F7">
-        <v>375</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -3674,7 +3674,7 @@
         <v>10</v>
       </c>
       <c r="F8">
-        <v>715</v>
+        <v>704</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -3694,7 +3694,7 @@
         <v>10</v>
       </c>
       <c r="F9">
-        <v>320</v>
+        <v>873</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -3714,7 +3714,7 @@
         <v>10</v>
       </c>
       <c r="F10">
-        <v>272</v>
+        <v>373</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -3734,7 +3734,7 @@
         <v>10</v>
       </c>
       <c r="F11">
-        <v>677</v>
+        <v>947</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -3754,7 +3754,7 @@
         <v>10</v>
       </c>
       <c r="F12">
-        <v>691</v>
+        <v>672</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -3774,7 +3774,7 @@
         <v>10</v>
       </c>
       <c r="F13">
-        <v>431</v>
+        <v>381</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -3794,7 +3794,7 @@
         <v>10</v>
       </c>
       <c r="F14">
-        <v>258</v>
+        <v>926</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -3814,7 +3814,7 @@
         <v>10</v>
       </c>
       <c r="F15">
-        <v>422</v>
+        <v>453</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -3834,7 +3834,7 @@
         <v>10</v>
       </c>
       <c r="F16">
-        <v>831</v>
+        <v>650</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -3854,7 +3854,7 @@
         <v>10</v>
       </c>
       <c r="F17">
-        <v>348</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -3874,7 +3874,7 @@
         <v>10</v>
       </c>
       <c r="F18">
-        <v>951</v>
+        <v>749</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -3894,7 +3894,7 @@
         <v>10</v>
       </c>
       <c r="F19">
-        <v>815</v>
+        <v>542</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -3914,7 +3914,7 @@
         <v>10</v>
       </c>
       <c r="F20">
-        <v>934</v>
+        <v>651</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -3934,7 +3934,7 @@
         <v>10</v>
       </c>
       <c r="F21">
-        <v>496</v>
+        <v>661</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -3954,7 +3954,7 @@
         <v>10</v>
       </c>
       <c r="F22">
-        <v>268</v>
+        <v>503</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -3974,7 +3974,7 @@
         <v>10</v>
       </c>
       <c r="F23">
-        <v>432</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -3994,7 +3994,7 @@
         <v>10</v>
       </c>
       <c r="F24">
-        <v>512</v>
+        <v>937</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -4014,7 +4014,7 @@
         <v>10</v>
       </c>
       <c r="F25">
-        <v>775</v>
+        <v>795</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -4034,7 +4034,7 @@
         <v>10</v>
       </c>
       <c r="F26">
-        <v>790</v>
+        <v>990</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -4054,7 +4054,7 @@
         <v>10</v>
       </c>
       <c r="F27">
-        <v>610</v>
+        <v>908</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -4074,7 +4074,7 @@
         <v>10</v>
       </c>
       <c r="F28">
-        <v>537</v>
+        <v>743</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -4094,7 +4094,7 @@
         <v>10</v>
       </c>
       <c r="F29">
-        <v>715</v>
+        <v>915</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -4114,7 +4114,7 @@
         <v>10</v>
       </c>
       <c r="F30">
-        <v>474</v>
+        <v>452</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -4134,7 +4134,7 @@
         <v>10</v>
       </c>
       <c r="F31">
-        <v>472</v>
+        <v>619</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -4154,7 +4154,7 @@
         <v>10</v>
       </c>
       <c r="F32">
-        <v>961</v>
+        <v>772</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -4174,7 +4174,7 @@
         <v>10</v>
       </c>
       <c r="F33">
-        <v>680</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -4194,7 +4194,7 @@
         <v>10</v>
       </c>
       <c r="F34">
-        <v>980</v>
+        <v>694</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -4214,7 +4214,7 @@
         <v>10</v>
       </c>
       <c r="F35">
-        <v>688</v>
+        <v>757</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -4234,7 +4234,7 @@
         <v>10</v>
       </c>
       <c r="F36">
-        <v>292</v>
+        <v>746</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -4254,7 +4254,7 @@
         <v>10</v>
       </c>
       <c r="F37">
-        <v>297</v>
+        <v>752</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -4274,7 +4274,7 @@
         <v>10</v>
       </c>
       <c r="F38">
-        <v>772</v>
+        <v>546</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>10</v>
       </c>
       <c r="F39">
-        <v>732</v>
+        <v>450</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -4314,7 +4314,7 @@
         <v>10</v>
       </c>
       <c r="F40">
-        <v>738</v>
+        <v>496</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -4334,7 +4334,7 @@
         <v>10</v>
       </c>
       <c r="F41">
-        <v>501</v>
+        <v>695</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -4354,7 +4354,7 @@
         <v>10</v>
       </c>
       <c r="F42">
-        <v>202</v>
+        <v>783</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -4374,7 +4374,7 @@
         <v>10</v>
       </c>
       <c r="F43">
-        <v>569</v>
+        <v>465</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -4394,7 +4394,7 @@
         <v>10</v>
       </c>
       <c r="F44">
-        <v>237</v>
+        <v>642</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -4414,7 +4414,7 @@
         <v>10</v>
       </c>
       <c r="F45">
-        <v>896</v>
+        <v>732</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -4434,7 +4434,7 @@
         <v>10</v>
       </c>
       <c r="F46">
-        <v>523</v>
+        <v>366</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -4454,7 +4454,7 @@
         <v>10</v>
       </c>
       <c r="F47">
-        <v>970</v>
+        <v>924</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -4474,7 +4474,7 @@
         <v>10</v>
       </c>
       <c r="F48">
-        <v>398</v>
+        <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -4494,7 +4494,7 @@
         <v>10</v>
       </c>
       <c r="F49">
-        <v>441</v>
+        <v>847</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -4514,7 +4514,7 @@
         <v>10</v>
       </c>
       <c r="F50">
-        <v>455</v>
+        <v>469</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -4534,7 +4534,7 @@
         <v>10</v>
       </c>
       <c r="F51">
-        <v>274</v>
+        <v>692</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -4554,7 +4554,7 @@
         <v>10</v>
       </c>
       <c r="F52">
-        <v>757</v>
+        <v>732</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -4574,7 +4574,7 @@
         <v>10</v>
       </c>
       <c r="F53">
-        <v>330</v>
+        <v>865</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -4594,7 +4594,7 @@
         <v>10</v>
       </c>
       <c r="F54">
-        <v>379</v>
+        <v>784</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -4614,7 +4614,7 @@
         <v>10</v>
       </c>
       <c r="F55">
-        <v>286</v>
+        <v>690</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -4634,7 +4634,7 @@
         <v>10</v>
       </c>
       <c r="F56">
-        <v>703</v>
+        <v>332</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -4654,7 +4654,7 @@
         <v>10</v>
       </c>
       <c r="F57">
-        <v>710</v>
+        <v>578</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -4674,7 +4674,7 @@
         <v>10</v>
       </c>
       <c r="F58">
-        <v>528</v>
+        <v>460</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -4694,7 +4694,7 @@
         <v>10</v>
       </c>
       <c r="F59">
-        <v>715</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -4714,7 +4714,7 @@
         <v>10</v>
       </c>
       <c r="F60">
-        <v>519</v>
+        <v>754</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -4734,7 +4734,7 @@
         <v>10</v>
       </c>
       <c r="F61">
-        <v>202</v>
+        <v>245</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -4754,7 +4754,7 @@
         <v>10</v>
       </c>
       <c r="F62">
-        <v>430</v>
+        <v>341</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -4774,7 +4774,7 @@
         <v>10</v>
       </c>
       <c r="F63">
-        <v>806</v>
+        <v>408</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -4794,7 +4794,7 @@
         <v>10</v>
       </c>
       <c r="F64">
-        <v>831</v>
+        <v>943</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -4814,7 +4814,7 @@
         <v>10</v>
       </c>
       <c r="F65">
-        <v>764</v>
+        <v>597</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -4834,7 +4834,7 @@
         <v>10</v>
       </c>
       <c r="F66">
-        <v>830</v>
+        <v>273</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -4854,7 +4854,7 @@
         <v>10</v>
       </c>
       <c r="F67">
-        <v>301</v>
+        <v>858</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>10</v>
       </c>
       <c r="F68">
-        <v>338</v>
+        <v>485</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -4894,7 +4894,7 @@
         <v>10</v>
       </c>
       <c r="F69">
-        <v>263</v>
+        <v>324</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -4914,7 +4914,7 @@
         <v>10</v>
       </c>
       <c r="F70">
-        <v>748</v>
+        <v>849</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -4934,7 +4934,7 @@
         <v>10</v>
       </c>
       <c r="F71">
-        <v>771</v>
+        <v>575</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -4954,7 +4954,7 @@
         <v>10</v>
       </c>
       <c r="F72">
-        <v>847</v>
+        <v>801</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -4974,7 +4974,7 @@
         <v>10</v>
       </c>
       <c r="F73">
-        <v>856</v>
+        <v>714</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -4994,7 +4994,7 @@
         <v>10</v>
       </c>
       <c r="F74">
-        <v>268</v>
+        <v>573</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -5014,7 +5014,7 @@
         <v>10</v>
       </c>
       <c r="F75">
-        <v>947</v>
+        <v>433</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -5034,7 +5034,7 @@
         <v>10</v>
       </c>
       <c r="F76">
-        <v>778</v>
+        <v>365</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -5054,7 +5054,7 @@
         <v>10</v>
       </c>
       <c r="F77">
-        <v>756</v>
+        <v>665</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -5074,7 +5074,7 @@
         <v>10</v>
       </c>
       <c r="F78">
-        <v>928</v>
+        <v>309</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -5094,7 +5094,7 @@
         <v>10</v>
       </c>
       <c r="F79">
-        <v>893</v>
+        <v>911</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -5114,7 +5114,7 @@
         <v>10</v>
       </c>
       <c r="F80">
-        <v>932</v>
+        <v>936</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -5134,7 +5134,7 @@
         <v>10</v>
       </c>
       <c r="F81">
-        <v>444</v>
+        <v>523</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -5154,7 +5154,7 @@
         <v>10</v>
       </c>
       <c r="F82">
-        <v>247</v>
+        <v>937</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -5174,7 +5174,7 @@
         <v>10</v>
       </c>
       <c r="F83">
-        <v>652</v>
+        <v>966</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -5194,7 +5194,7 @@
         <v>10</v>
       </c>
       <c r="F84">
-        <v>802</v>
+        <v>606</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -5214,7 +5214,7 @@
         <v>10</v>
       </c>
       <c r="F85">
-        <v>303</v>
+        <v>513</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -5234,7 +5234,7 @@
         <v>10</v>
       </c>
       <c r="F86">
-        <v>971</v>
+        <v>786</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -5254,7 +5254,7 @@
         <v>10</v>
       </c>
       <c r="F87">
-        <v>788</v>
+        <v>718</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -5274,7 +5274,7 @@
         <v>10</v>
       </c>
       <c r="F88">
-        <v>707</v>
+        <v>894</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -5294,7 +5294,7 @@
         <v>10</v>
       </c>
       <c r="F89">
-        <v>842</v>
+        <v>999</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -5314,7 +5314,7 @@
         <v>10</v>
       </c>
       <c r="F90">
-        <v>845</v>
+        <v>645</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -5334,7 +5334,7 @@
         <v>10</v>
       </c>
       <c r="F91">
-        <v>244</v>
+        <v>458</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -5354,7 +5354,7 @@
         <v>10</v>
       </c>
       <c r="F92">
-        <v>871</v>
+        <v>378</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -5374,7 +5374,7 @@
         <v>10</v>
       </c>
       <c r="F93">
-        <v>338</v>
+        <v>356</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -5394,7 +5394,7 @@
         <v>10</v>
       </c>
       <c r="F94">
-        <v>780</v>
+        <v>772</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -5414,7 +5414,7 @@
         <v>10</v>
       </c>
       <c r="F95">
-        <v>936</v>
+        <v>367</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -5434,7 +5434,7 @@
         <v>10</v>
       </c>
       <c r="F96">
-        <v>387</v>
+        <v>823</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>10</v>
       </c>
       <c r="F97">
-        <v>739</v>
+        <v>427</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -5474,7 +5474,7 @@
         <v>10</v>
       </c>
       <c r="F98">
-        <v>414</v>
+        <v>363</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -5494,7 +5494,7 @@
         <v>10</v>
       </c>
       <c r="F99">
-        <v>558</v>
+        <v>923</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -5514,7 +5514,7 @@
         <v>10</v>
       </c>
       <c r="F100">
-        <v>690</v>
+        <v>448</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -5534,7 +5534,7 @@
         <v>10</v>
       </c>
       <c r="F101">
-        <v>225</v>
+        <v>456</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -5554,7 +5554,7 @@
         <v>10</v>
       </c>
       <c r="F102">
-        <v>725</v>
+        <v>763</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -5574,7 +5574,7 @@
         <v>10</v>
       </c>
       <c r="F103">
-        <v>418</v>
+        <v>785</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -5594,7 +5594,7 @@
         <v>10</v>
       </c>
       <c r="F104">
-        <v>595</v>
+        <v>880</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -5614,7 +5614,7 @@
         <v>10</v>
       </c>
       <c r="F105">
-        <v>346</v>
+        <v>964</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -5634,7 +5634,7 @@
         <v>10</v>
       </c>
       <c r="F106">
-        <v>928</v>
+        <v>629</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -5654,7 +5654,7 @@
         <v>10</v>
       </c>
       <c r="F107">
-        <v>704</v>
+        <v>250</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -5674,7 +5674,7 @@
         <v>10</v>
       </c>
       <c r="F108">
-        <v>261</v>
+        <v>627</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -5694,7 +5694,7 @@
         <v>10</v>
       </c>
       <c r="F109">
-        <v>859</v>
+        <v>426</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -5714,7 +5714,7 @@
         <v>10</v>
       </c>
       <c r="F110">
-        <v>979</v>
+        <v>467</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -5734,7 +5734,7 @@
         <v>10</v>
       </c>
       <c r="F111">
-        <v>370</v>
+        <v>546</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -5754,7 +5754,7 @@
         <v>10</v>
       </c>
       <c r="F112">
-        <v>556</v>
+        <v>202</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -5774,7 +5774,7 @@
         <v>10</v>
       </c>
       <c r="F113">
-        <v>565</v>
+        <v>549</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -5794,7 +5794,7 @@
         <v>10</v>
       </c>
       <c r="F114">
-        <v>787</v>
+        <v>477</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -5814,7 +5814,7 @@
         <v>10</v>
       </c>
       <c r="F115">
-        <v>309</v>
+        <v>968</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -5834,7 +5834,7 @@
         <v>10</v>
       </c>
       <c r="F116">
-        <v>370</v>
+        <v>576</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -5854,7 +5854,7 @@
         <v>10</v>
       </c>
       <c r="F117">
-        <v>346</v>
+        <v>782</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -5874,7 +5874,7 @@
         <v>10</v>
       </c>
       <c r="F118">
-        <v>742</v>
+        <v>729</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -5894,7 +5894,7 @@
         <v>10</v>
       </c>
       <c r="F119">
-        <v>344</v>
+        <v>814</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -5914,7 +5914,7 @@
         <v>10</v>
       </c>
       <c r="F120">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -5934,7 +5934,7 @@
         <v>10</v>
       </c>
       <c r="F121">
-        <v>562</v>
+        <v>828</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -5954,7 +5954,7 @@
         <v>10</v>
       </c>
       <c r="F122">
-        <v>607</v>
+        <v>292</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -5974,7 +5974,7 @@
         <v>10</v>
       </c>
       <c r="F123">
-        <v>441</v>
+        <v>685</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -5994,7 +5994,7 @@
         <v>10</v>
       </c>
       <c r="F124">
-        <v>286</v>
+        <v>419</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -6014,7 +6014,7 @@
         <v>10</v>
       </c>
       <c r="F125">
-        <v>582</v>
+        <v>269</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>10</v>
       </c>
       <c r="F126">
-        <v>374</v>
+        <v>717</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -6054,7 +6054,7 @@
         <v>10</v>
       </c>
       <c r="F127">
-        <v>282</v>
+        <v>556</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -6074,7 +6074,7 @@
         <v>10</v>
       </c>
       <c r="F128">
-        <v>380</v>
+        <v>934</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -6094,7 +6094,7 @@
         <v>10</v>
       </c>
       <c r="F129">
-        <v>263</v>
+        <v>449</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -6114,7 +6114,7 @@
         <v>10</v>
       </c>
       <c r="F130">
-        <v>379</v>
+        <v>871</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -6134,7 +6134,7 @@
         <v>10</v>
       </c>
       <c r="F131">
-        <v>927</v>
+        <v>382</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -6154,7 +6154,7 @@
         <v>10</v>
       </c>
       <c r="F132">
-        <v>631</v>
+        <v>677</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -6174,7 +6174,7 @@
         <v>10</v>
       </c>
       <c r="F133">
-        <v>711</v>
+        <v>323</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -6194,7 +6194,7 @@
         <v>10</v>
       </c>
       <c r="F134">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -6214,7 +6214,7 @@
         <v>10</v>
       </c>
       <c r="F135">
-        <v>493</v>
+        <v>516</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -6234,7 +6234,7 @@
         <v>10</v>
       </c>
       <c r="F136">
-        <v>836</v>
+        <v>677</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -6254,7 +6254,7 @@
         <v>10</v>
       </c>
       <c r="F137">
-        <v>276</v>
+        <v>384</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -6274,7 +6274,7 @@
         <v>10</v>
       </c>
       <c r="F138">
-        <v>250</v>
+        <v>340</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -6294,7 +6294,7 @@
         <v>10</v>
       </c>
       <c r="F139">
-        <v>568</v>
+        <v>249</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
@@ -6314,7 +6314,7 @@
         <v>10</v>
       </c>
       <c r="F140">
-        <v>689</v>
+        <v>612</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
@@ -6334,7 +6334,7 @@
         <v>10</v>
       </c>
       <c r="F141">
-        <v>481</v>
+        <v>800</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
@@ -6354,7 +6354,7 @@
         <v>10</v>
       </c>
       <c r="F142">
-        <v>496</v>
+        <v>359</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
@@ -6374,7 +6374,7 @@
         <v>10</v>
       </c>
       <c r="F143">
-        <v>435</v>
+        <v>595</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
@@ -6394,7 +6394,7 @@
         <v>10</v>
       </c>
       <c r="F144">
-        <v>353</v>
+        <v>454</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
@@ -6414,7 +6414,7 @@
         <v>10</v>
       </c>
       <c r="F145">
-        <v>953</v>
+        <v>914</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
@@ -6434,7 +6434,7 @@
         <v>10</v>
       </c>
       <c r="F146">
-        <v>550</v>
+        <v>290</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -6454,7 +6454,7 @@
         <v>10</v>
       </c>
       <c r="F147">
-        <v>502</v>
+        <v>740</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -6474,7 +6474,7 @@
         <v>10</v>
       </c>
       <c r="F148">
-        <v>240</v>
+        <v>468</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
@@ -6494,7 +6494,7 @@
         <v>10</v>
       </c>
       <c r="F149">
-        <v>820</v>
+        <v>397</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
@@ -6514,7 +6514,7 @@
         <v>10</v>
       </c>
       <c r="F150">
-        <v>359</v>
+        <v>772</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -6534,7 +6534,7 @@
         <v>10</v>
       </c>
       <c r="F151">
-        <v>351</v>
+        <v>585</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
@@ -6554,7 +6554,7 @@
         <v>10</v>
       </c>
       <c r="F152">
-        <v>770</v>
+        <v>795</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -6574,7 +6574,7 @@
         <v>10</v>
       </c>
       <c r="F153">
-        <v>772</v>
+        <v>614</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
@@ -6594,7 +6594,7 @@
         <v>10</v>
       </c>
       <c r="F154">
-        <v>421</v>
+        <v>800</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>10</v>
       </c>
       <c r="F155">
-        <v>244</v>
+        <v>625</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
@@ -6634,7 +6634,7 @@
         <v>10</v>
       </c>
       <c r="F156">
-        <v>447</v>
+        <v>213</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
@@ -6654,7 +6654,7 @@
         <v>10</v>
       </c>
       <c r="F157">
-        <v>846</v>
+        <v>359</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
@@ -6674,7 +6674,7 @@
         <v>10</v>
       </c>
       <c r="F158">
-        <v>783</v>
+        <v>828</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
@@ -6694,7 +6694,7 @@
         <v>10</v>
       </c>
       <c r="F159">
-        <v>914</v>
+        <v>666</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
@@ -6714,7 +6714,7 @@
         <v>10</v>
       </c>
       <c r="F160">
-        <v>267</v>
+        <v>696</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
@@ -6734,7 +6734,7 @@
         <v>10</v>
       </c>
       <c r="F161">
-        <v>292</v>
+        <v>591</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
@@ -6754,7 +6754,7 @@
         <v>10</v>
       </c>
       <c r="F162">
-        <v>796</v>
+        <v>366</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
@@ -6774,7 +6774,7 @@
         <v>10</v>
       </c>
       <c r="F163">
-        <v>369</v>
+        <v>678</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
@@ -6794,7 +6794,7 @@
         <v>10</v>
       </c>
       <c r="F164">
-        <v>424</v>
+        <v>409</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
@@ -6814,7 +6814,7 @@
         <v>10</v>
       </c>
       <c r="F165">
-        <v>760</v>
+        <v>641</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
@@ -6834,7 +6834,7 @@
         <v>10</v>
       </c>
       <c r="F166">
-        <v>693</v>
+        <v>349</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
@@ -6854,7 +6854,7 @@
         <v>10</v>
       </c>
       <c r="F167">
-        <v>845</v>
+        <v>888</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
@@ -6874,7 +6874,7 @@
         <v>10</v>
       </c>
       <c r="F168">
-        <v>860</v>
+        <v>659</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
@@ -6894,7 +6894,7 @@
         <v>10</v>
       </c>
       <c r="F169">
-        <v>887</v>
+        <v>364</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
@@ -6914,7 +6914,7 @@
         <v>10</v>
       </c>
       <c r="F170">
-        <v>522</v>
+        <v>630</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
@@ -6934,7 +6934,7 @@
         <v>10</v>
       </c>
       <c r="F171">
-        <v>202</v>
+        <v>564</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
@@ -6954,7 +6954,7 @@
         <v>10</v>
       </c>
       <c r="F172">
-        <v>410</v>
+        <v>973</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
@@ -6974,7 +6974,7 @@
         <v>10</v>
       </c>
       <c r="F173">
-        <v>457</v>
+        <v>884</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
@@ -6994,7 +6994,7 @@
         <v>10</v>
       </c>
       <c r="F174">
-        <v>882</v>
+        <v>584</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
@@ -7014,7 +7014,7 @@
         <v>10</v>
       </c>
       <c r="F175">
-        <v>909</v>
+        <v>930</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
@@ -7034,7 +7034,7 @@
         <v>10</v>
       </c>
       <c r="F176">
-        <v>764</v>
+        <v>872</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
@@ -7054,7 +7054,7 @@
         <v>10</v>
       </c>
       <c r="F177">
-        <v>411</v>
+        <v>286</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
@@ -7074,7 +7074,7 @@
         <v>10</v>
       </c>
       <c r="F178">
-        <v>987</v>
+        <v>682</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
@@ -7094,7 +7094,7 @@
         <v>10</v>
       </c>
       <c r="F179">
-        <v>805</v>
+        <v>277</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
@@ -7114,7 +7114,7 @@
         <v>10</v>
       </c>
       <c r="F180">
-        <v>896</v>
+        <v>482</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
@@ -7134,7 +7134,7 @@
         <v>10</v>
       </c>
       <c r="F181">
-        <v>369</v>
+        <v>418</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
@@ -7154,7 +7154,7 @@
         <v>10</v>
       </c>
       <c r="F182">
-        <v>572</v>
+        <v>243</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
@@ -7174,7 +7174,7 @@
         <v>10</v>
       </c>
       <c r="F183">
-        <v>443</v>
+        <v>221</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>10</v>
       </c>
       <c r="F184">
-        <v>891</v>
+        <v>758</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
@@ -7214,7 +7214,7 @@
         <v>10</v>
       </c>
       <c r="F185">
-        <v>945</v>
+        <v>745</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
@@ -7234,7 +7234,7 @@
         <v>10</v>
       </c>
       <c r="F186">
-        <v>961</v>
+        <v>662</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
@@ -7254,7 +7254,7 @@
         <v>10</v>
       </c>
       <c r="F187">
-        <v>734</v>
+        <v>653</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
@@ -7274,7 +7274,7 @@
         <v>10</v>
       </c>
       <c r="F188">
-        <v>948</v>
+        <v>657</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
@@ -7294,7 +7294,7 @@
         <v>10</v>
       </c>
       <c r="F189">
-        <v>769</v>
+        <v>696</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
@@ -7314,7 +7314,7 @@
         <v>10</v>
       </c>
       <c r="F190">
-        <v>220</v>
+        <v>206</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
@@ -7334,7 +7334,7 @@
         <v>10</v>
       </c>
       <c r="F191">
-        <v>631</v>
+        <v>579</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
@@ -7354,7 +7354,7 @@
         <v>10</v>
       </c>
       <c r="F192">
-        <v>570</v>
+        <v>559</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
@@ -7374,7 +7374,7 @@
         <v>10</v>
       </c>
       <c r="F193">
-        <v>222</v>
+        <v>777</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
@@ -7394,7 +7394,7 @@
         <v>10</v>
       </c>
       <c r="F194">
-        <v>916</v>
+        <v>538</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
@@ -7414,7 +7414,7 @@
         <v>10</v>
       </c>
       <c r="F195">
-        <v>675</v>
+        <v>669</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
@@ -7434,7 +7434,7 @@
         <v>10</v>
       </c>
       <c r="F196">
-        <v>303</v>
+        <v>707</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
@@ -7454,7 +7454,7 @@
         <v>10</v>
       </c>
       <c r="F197">
-        <v>949</v>
+        <v>666</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
@@ -7474,7 +7474,7 @@
         <v>10</v>
       </c>
       <c r="F198">
-        <v>946</v>
+        <v>539</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
@@ -7494,7 +7494,7 @@
         <v>10</v>
       </c>
       <c r="F199">
-        <v>296</v>
+        <v>610</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
@@ -7514,7 +7514,7 @@
         <v>10</v>
       </c>
       <c r="F200">
-        <v>352</v>
+        <v>959</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
@@ -7534,7 +7534,7 @@
         <v>10</v>
       </c>
       <c r="F201">
-        <v>364</v>
+        <v>219</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
@@ -7554,7 +7554,7 @@
         <v>10</v>
       </c>
       <c r="F202">
-        <v>620</v>
+        <v>663</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
@@ -7574,7 +7574,7 @@
         <v>10</v>
       </c>
       <c r="F203">
-        <v>991</v>
+        <v>295</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
@@ -7594,7 +7594,7 @@
         <v>10</v>
       </c>
       <c r="F204">
-        <v>667</v>
+        <v>730</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
@@ -7614,7 +7614,7 @@
         <v>10</v>
       </c>
       <c r="F205">
-        <v>211</v>
+        <v>951</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
@@ -7634,7 +7634,7 @@
         <v>10</v>
       </c>
       <c r="F206">
-        <v>239</v>
+        <v>436</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
@@ -7654,7 +7654,7 @@
         <v>10</v>
       </c>
       <c r="F207">
-        <v>821</v>
+        <v>904</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
@@ -7674,7 +7674,7 @@
         <v>10</v>
       </c>
       <c r="F208">
-        <v>970</v>
+        <v>833</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
@@ -7694,7 +7694,7 @@
         <v>10</v>
       </c>
       <c r="F209">
-        <v>649</v>
+        <v>889</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
@@ -7714,7 +7714,7 @@
         <v>10</v>
       </c>
       <c r="F210">
-        <v>694</v>
+        <v>401</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
@@ -7734,7 +7734,7 @@
         <v>10</v>
       </c>
       <c r="F211">
-        <v>949</v>
+        <v>716</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
@@ -7754,7 +7754,7 @@
         <v>10</v>
       </c>
       <c r="F212">
-        <v>619</v>
+        <v>484</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>10</v>
       </c>
       <c r="F213">
-        <v>791</v>
+        <v>325</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
@@ -7794,7 +7794,7 @@
         <v>10</v>
       </c>
       <c r="F214">
-        <v>726</v>
+        <v>862</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
@@ -7814,7 +7814,7 @@
         <v>10</v>
       </c>
       <c r="F215">
-        <v>261</v>
+        <v>992</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
@@ -7834,7 +7834,7 @@
         <v>10</v>
       </c>
       <c r="F216">
-        <v>892</v>
+        <v>835</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
@@ -7854,7 +7854,7 @@
         <v>10</v>
       </c>
       <c r="F217">
-        <v>760</v>
+        <v>876</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
@@ -7874,7 +7874,7 @@
         <v>10</v>
       </c>
       <c r="F218">
-        <v>443</v>
+        <v>471</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
@@ -7894,7 +7894,7 @@
         <v>10</v>
       </c>
       <c r="F219">
-        <v>850</v>
+        <v>729</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
@@ -7914,7 +7914,7 @@
         <v>10</v>
       </c>
       <c r="F220">
-        <v>273</v>
+        <v>297</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
@@ -7934,7 +7934,7 @@
         <v>10</v>
       </c>
       <c r="F221">
-        <v>810</v>
+        <v>510</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
@@ -7954,7 +7954,7 @@
         <v>10</v>
       </c>
       <c r="F222">
-        <v>241</v>
+        <v>512</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
@@ -7974,7 +7974,7 @@
         <v>10</v>
       </c>
       <c r="F223">
-        <v>961</v>
+        <v>267</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
@@ -7994,7 +7994,7 @@
         <v>10</v>
       </c>
       <c r="F224">
-        <v>383</v>
+        <v>979</v>
       </c>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.25">
@@ -8014,7 +8014,7 @@
         <v>10</v>
       </c>
       <c r="F225">
-        <v>806</v>
+        <v>951</v>
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.25">
@@ -8034,7 +8034,7 @@
         <v>10</v>
       </c>
       <c r="F226">
-        <v>938</v>
+        <v>396</v>
       </c>
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.25">
@@ -8054,7 +8054,7 @@
         <v>10</v>
       </c>
       <c r="F227">
-        <v>493</v>
+        <v>858</v>
       </c>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.25">
@@ -8074,7 +8074,7 @@
         <v>10</v>
       </c>
       <c r="F228">
-        <v>397</v>
+        <v>239</v>
       </c>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.25">
@@ -8094,7 +8094,7 @@
         <v>10</v>
       </c>
       <c r="F229">
-        <v>423</v>
+        <v>379</v>
       </c>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.25">
@@ -8114,7 +8114,7 @@
         <v>10</v>
       </c>
       <c r="F230">
-        <v>740</v>
+        <v>541</v>
       </c>
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.25">
@@ -8134,7 +8134,7 @@
         <v>10</v>
       </c>
       <c r="F231">
-        <v>403</v>
+        <v>370</v>
       </c>
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.25">
@@ -8154,7 +8154,7 @@
         <v>10</v>
       </c>
       <c r="F232">
-        <v>806</v>
+        <v>938</v>
       </c>
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.25">
@@ -8174,7 +8174,7 @@
         <v>10</v>
       </c>
       <c r="F233">
-        <v>763</v>
+        <v>801</v>
       </c>
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.25">
@@ -8194,7 +8194,7 @@
         <v>10</v>
       </c>
       <c r="F234">
-        <v>657</v>
+        <v>583</v>
       </c>
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.25">
@@ -8214,7 +8214,7 @@
         <v>10</v>
       </c>
       <c r="F235">
-        <v>240</v>
+        <v>452</v>
       </c>
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.25">
@@ -8234,7 +8234,7 @@
         <v>10</v>
       </c>
       <c r="F236">
-        <v>539</v>
+        <v>943</v>
       </c>
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.25">
@@ -8254,7 +8254,7 @@
         <v>10</v>
       </c>
       <c r="F237">
-        <v>984</v>
+        <v>289</v>
       </c>
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.25">
@@ -8274,7 +8274,7 @@
         <v>10</v>
       </c>
       <c r="F238">
-        <v>551</v>
+        <v>390</v>
       </c>
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.25">
@@ -8294,7 +8294,7 @@
         <v>10</v>
       </c>
       <c r="F239">
-        <v>455</v>
+        <v>963</v>
       </c>
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.25">
@@ -8314,7 +8314,7 @@
         <v>10</v>
       </c>
       <c r="F240">
-        <v>524</v>
+        <v>930</v>
       </c>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.25">
@@ -8334,7 +8334,7 @@
         <v>10</v>
       </c>
       <c r="F241">
-        <v>734</v>
+        <v>904</v>
       </c>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>10</v>
       </c>
       <c r="F242">
-        <v>589</v>
+        <v>783</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.25">
@@ -8374,7 +8374,7 @@
         <v>10</v>
       </c>
       <c r="F243">
-        <v>787</v>
+        <v>362</v>
       </c>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.25">
@@ -8394,7 +8394,7 @@
         <v>10</v>
       </c>
       <c r="F244">
-        <v>869</v>
+        <v>659</v>
       </c>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.25">
@@ -8414,7 +8414,7 @@
         <v>10</v>
       </c>
       <c r="F245">
-        <v>740</v>
+        <v>612</v>
       </c>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.25">
@@ -8434,7 +8434,7 @@
         <v>10</v>
       </c>
       <c r="F246">
-        <v>761</v>
+        <v>851</v>
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.25">
@@ -8454,7 +8454,7 @@
         <v>10</v>
       </c>
       <c r="F247">
-        <v>366</v>
+        <v>355</v>
       </c>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.25">
@@ -8474,7 +8474,7 @@
         <v>10</v>
       </c>
       <c r="F248">
-        <v>880</v>
+        <v>868</v>
       </c>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.25">
@@ -8494,7 +8494,7 @@
         <v>10</v>
       </c>
       <c r="F249">
-        <v>252</v>
+        <v>837</v>
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.25">
@@ -8514,7 +8514,7 @@
         <v>10</v>
       </c>
       <c r="F250">
-        <v>235</v>
+        <v>386</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.25">
@@ -8534,7 +8534,7 @@
         <v>10</v>
       </c>
       <c r="F251">
-        <v>421</v>
+        <v>337</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.25">
@@ -8554,7 +8554,7 @@
         <v>10</v>
       </c>
       <c r="F252">
-        <v>273</v>
+        <v>676</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.25">
@@ -8574,7 +8574,7 @@
         <v>10</v>
       </c>
       <c r="F253">
-        <v>445</v>
+        <v>464</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.25">
@@ -8594,7 +8594,7 @@
         <v>10</v>
       </c>
       <c r="F254">
-        <v>497</v>
+        <v>938</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.25">
@@ -8614,7 +8614,7 @@
         <v>10</v>
       </c>
       <c r="F255">
-        <v>306</v>
+        <v>658</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.25">
@@ -8634,7 +8634,7 @@
         <v>10</v>
       </c>
       <c r="F256">
-        <v>990</v>
+        <v>397</v>
       </c>
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.25">
@@ -8654,7 +8654,7 @@
         <v>10</v>
       </c>
       <c r="F257">
-        <v>608</v>
+        <v>358</v>
       </c>
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.25">
@@ -8674,7 +8674,7 @@
         <v>10</v>
       </c>
       <c r="F258">
-        <v>914</v>
+        <v>377</v>
       </c>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.25">
@@ -8694,7 +8694,7 @@
         <v>10</v>
       </c>
       <c r="F259">
-        <v>758</v>
+        <v>909</v>
       </c>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.25">
@@ -8714,7 +8714,7 @@
         <v>10</v>
       </c>
       <c r="F260">
-        <v>458</v>
+        <v>502</v>
       </c>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.25">
@@ -8734,7 +8734,7 @@
         <v>10</v>
       </c>
       <c r="F261">
-        <v>624</v>
+        <v>338</v>
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.25">
@@ -8754,7 +8754,7 @@
         <v>10</v>
       </c>
       <c r="F262">
-        <v>227</v>
+        <v>958</v>
       </c>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.25">
@@ -8774,7 +8774,7 @@
         <v>10</v>
       </c>
       <c r="F263">
-        <v>235</v>
+        <v>645</v>
       </c>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.25">
@@ -8794,7 +8794,7 @@
         <v>10</v>
       </c>
       <c r="F264">
-        <v>898</v>
+        <v>712</v>
       </c>
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.25">
@@ -8814,7 +8814,7 @@
         <v>10</v>
       </c>
       <c r="F265">
-        <v>248</v>
+        <v>701</v>
       </c>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.25">
@@ -8834,7 +8834,7 @@
         <v>10</v>
       </c>
       <c r="F266">
-        <v>290</v>
+        <v>842</v>
       </c>
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.25">
@@ -8854,7 +8854,7 @@
         <v>10</v>
       </c>
       <c r="F267">
-        <v>838</v>
+        <v>800</v>
       </c>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.25">
@@ -8874,7 +8874,7 @@
         <v>10</v>
       </c>
       <c r="F268">
-        <v>673</v>
+        <v>267</v>
       </c>
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.25">
@@ -8894,7 +8894,7 @@
         <v>10</v>
       </c>
       <c r="F269">
-        <v>995</v>
+        <v>981</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.25">
@@ -8914,7 +8914,7 @@
         <v>10</v>
       </c>
       <c r="F270">
-        <v>540</v>
+        <v>575</v>
       </c>
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>10</v>
       </c>
       <c r="F271">
-        <v>633</v>
+        <v>936</v>
       </c>
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.25">
@@ -8954,7 +8954,7 @@
         <v>10</v>
       </c>
       <c r="F272">
-        <v>224</v>
+        <v>984</v>
       </c>
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.25">
@@ -8974,7 +8974,7 @@
         <v>10</v>
       </c>
       <c r="F273">
-        <v>333</v>
+        <v>943</v>
       </c>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.25">
@@ -8994,7 +8994,7 @@
         <v>10</v>
       </c>
       <c r="F274">
-        <v>429</v>
+        <v>800</v>
       </c>
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.25">
@@ -9014,7 +9014,7 @@
         <v>10</v>
       </c>
       <c r="F275">
-        <v>961</v>
+        <v>434</v>
       </c>
     </row>
     <row r="276" spans="1:6" x14ac:dyDescent="0.25">
@@ -9034,7 +9034,7 @@
         <v>10</v>
       </c>
       <c r="F276">
-        <v>717</v>
+        <v>411</v>
       </c>
     </row>
     <row r="277" spans="1:6" x14ac:dyDescent="0.25">
@@ -9054,7 +9054,7 @@
         <v>10</v>
       </c>
       <c r="F277">
-        <v>934</v>
+        <v>922</v>
       </c>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.25">
@@ -9074,7 +9074,7 @@
         <v>10</v>
       </c>
       <c r="F278">
-        <v>809</v>
+        <v>460</v>
       </c>
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.25">
@@ -9094,7 +9094,7 @@
         <v>10</v>
       </c>
       <c r="F279">
-        <v>629</v>
+        <v>297</v>
       </c>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.25">
@@ -9114,7 +9114,7 @@
         <v>10</v>
       </c>
       <c r="F280">
-        <v>599</v>
+        <v>501</v>
       </c>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.25">
@@ -9134,7 +9134,7 @@
         <v>10</v>
       </c>
       <c r="F281">
-        <v>989</v>
+        <v>488</v>
       </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.25">
@@ -9154,7 +9154,7 @@
         <v>10</v>
       </c>
       <c r="F282">
-        <v>388</v>
+        <v>837</v>
       </c>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.25">
@@ -9174,7 +9174,7 @@
         <v>10</v>
       </c>
       <c r="F283">
-        <v>226</v>
+        <v>318</v>
       </c>
     </row>
     <row r="284" spans="1:6" x14ac:dyDescent="0.25">
@@ -9194,7 +9194,7 @@
         <v>10</v>
       </c>
       <c r="F284">
-        <v>841</v>
+        <v>284</v>
       </c>
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.25">
@@ -9214,7 +9214,7 @@
         <v>10</v>
       </c>
       <c r="F285">
-        <v>433</v>
+        <v>806</v>
       </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.25">
@@ -9234,7 +9234,7 @@
         <v>10</v>
       </c>
       <c r="F286">
-        <v>953</v>
+        <v>319</v>
       </c>
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.25">
@@ -9254,7 +9254,7 @@
         <v>10</v>
       </c>
       <c r="F287">
-        <v>605</v>
+        <v>576</v>
       </c>
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.25">
@@ -9274,7 +9274,7 @@
         <v>10</v>
       </c>
       <c r="F288">
-        <v>277</v>
+        <v>656</v>
       </c>
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.25">
@@ -9294,7 +9294,7 @@
         <v>10</v>
       </c>
       <c r="F289">
-        <v>558</v>
+        <v>207</v>
       </c>
     </row>
     <row r="290" spans="1:6" x14ac:dyDescent="0.25">
@@ -9314,7 +9314,7 @@
         <v>10</v>
       </c>
       <c r="F290">
-        <v>552</v>
+        <v>233</v>
       </c>
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.25">
@@ -9334,7 +9334,7 @@
         <v>10</v>
       </c>
       <c r="F291">
-        <v>277</v>
+        <v>688</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.25">
@@ -9354,7 +9354,7 @@
         <v>10</v>
       </c>
       <c r="F292">
-        <v>730</v>
+        <v>296</v>
       </c>
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.25">
@@ -9374,7 +9374,7 @@
         <v>10</v>
       </c>
       <c r="F293">
-        <v>530</v>
+        <v>414</v>
       </c>
     </row>
     <row r="294" spans="1:6" x14ac:dyDescent="0.25">
@@ -9394,7 +9394,7 @@
         <v>10</v>
       </c>
       <c r="F294">
-        <v>454</v>
+        <v>704</v>
       </c>
     </row>
     <row r="295" spans="1:6" x14ac:dyDescent="0.25">
@@ -9414,7 +9414,7 @@
         <v>10</v>
       </c>
       <c r="F295">
-        <v>529</v>
+        <v>694</v>
       </c>
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.25">
@@ -9434,7 +9434,7 @@
         <v>10</v>
       </c>
       <c r="F296">
-        <v>276</v>
+        <v>378</v>
       </c>
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.25">
@@ -9454,7 +9454,7 @@
         <v>10</v>
       </c>
       <c r="F297">
-        <v>669</v>
+        <v>950</v>
       </c>
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.25">
@@ -9474,7 +9474,7 @@
         <v>10</v>
       </c>
       <c r="F298">
-        <v>223</v>
+        <v>902</v>
       </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.25">
@@ -9494,7 +9494,7 @@
         <v>10</v>
       </c>
       <c r="F299">
-        <v>677</v>
+        <v>789</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>10</v>
       </c>
       <c r="F300">
-        <v>328</v>
+        <v>766</v>
       </c>
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.25">
@@ -9534,7 +9534,7 @@
         <v>10</v>
       </c>
       <c r="F301">
-        <v>705</v>
+        <v>971</v>
       </c>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.25">
@@ -9554,7 +9554,7 @@
         <v>10</v>
       </c>
       <c r="F302">
-        <v>384</v>
+        <v>425</v>
       </c>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.25">
@@ -9574,7 +9574,7 @@
         <v>10</v>
       </c>
       <c r="F303">
-        <v>868</v>
+        <v>900</v>
       </c>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.25">
@@ -9594,7 +9594,7 @@
         <v>10</v>
       </c>
       <c r="F304">
-        <v>238</v>
+        <v>968</v>
       </c>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.25">
@@ -9614,7 +9614,7 @@
         <v>10</v>
       </c>
       <c r="F305">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.25">
@@ -9634,7 +9634,7 @@
         <v>10</v>
       </c>
       <c r="F306">
-        <v>379</v>
+        <v>247</v>
       </c>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.25">
@@ -9654,7 +9654,7 @@
         <v>10</v>
       </c>
       <c r="F307">
-        <v>745</v>
+        <v>986</v>
       </c>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.25">
@@ -9674,7 +9674,7 @@
         <v>10</v>
       </c>
       <c r="F308">
-        <v>909</v>
+        <v>505</v>
       </c>
     </row>
     <row r="309" spans="1:6" x14ac:dyDescent="0.25">
@@ -9694,7 +9694,7 @@
         <v>10</v>
       </c>
       <c r="F309">
-        <v>795</v>
+        <v>749</v>
       </c>
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.25">
@@ -9714,7 +9714,7 @@
         <v>10</v>
       </c>
       <c r="F310">
-        <v>946</v>
+        <v>825</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.25">
@@ -9734,7 +9734,7 @@
         <v>10</v>
       </c>
       <c r="F311">
-        <v>695</v>
+        <v>902</v>
       </c>
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.25">
@@ -9754,7 +9754,7 @@
         <v>10</v>
       </c>
       <c r="F312">
-        <v>258</v>
+        <v>732</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.25">
@@ -9774,7 +9774,7 @@
         <v>10</v>
       </c>
       <c r="F313">
-        <v>556</v>
+        <v>830</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.25">
@@ -9794,7 +9794,7 @@
         <v>10</v>
       </c>
       <c r="F314">
-        <v>846</v>
+        <v>606</v>
       </c>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.25">
@@ -9814,7 +9814,7 @@
         <v>10</v>
       </c>
       <c r="F315">
-        <v>915</v>
+        <v>212</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.25">
@@ -9834,7 +9834,7 @@
         <v>10</v>
       </c>
       <c r="F316">
-        <v>330</v>
+        <v>961</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.25">
@@ -9854,7 +9854,7 @@
         <v>10</v>
       </c>
       <c r="F317">
-        <v>243</v>
+        <v>304</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.25">
@@ -9874,7 +9874,7 @@
         <v>10</v>
       </c>
       <c r="F318">
-        <v>215</v>
+        <v>854</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.25">
@@ -9894,7 +9894,7 @@
         <v>10</v>
       </c>
       <c r="F319">
-        <v>614</v>
+        <v>893</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -9914,7 +9914,7 @@
         <v>10</v>
       </c>
       <c r="F320">
-        <v>446</v>
+        <v>736</v>
       </c>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.25">
@@ -9934,7 +9934,7 @@
         <v>10</v>
       </c>
       <c r="F321">
-        <v>886</v>
+        <v>517</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.25">
@@ -9954,7 +9954,7 @@
         <v>10</v>
       </c>
       <c r="F322">
-        <v>446</v>
+        <v>794</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.25">
@@ -9974,7 +9974,7 @@
         <v>10</v>
       </c>
       <c r="F323">
-        <v>763</v>
+        <v>319</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.25">
@@ -9994,7 +9994,7 @@
         <v>10</v>
       </c>
       <c r="F324">
-        <v>513</v>
+        <v>669</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.25">
@@ -10014,7 +10014,7 @@
         <v>10</v>
       </c>
       <c r="F325">
-        <v>524</v>
+        <v>611</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.25">
@@ -10034,7 +10034,7 @@
         <v>10</v>
       </c>
       <c r="F326">
-        <v>918</v>
+        <v>363</v>
       </c>
     </row>
     <row r="327" spans="1:6" x14ac:dyDescent="0.25">
@@ -10054,7 +10054,7 @@
         <v>10</v>
       </c>
       <c r="F327">
-        <v>560</v>
+        <v>238</v>
       </c>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.25">
@@ -10074,7 +10074,7 @@
         <v>10</v>
       </c>
       <c r="F328">
-        <v>955</v>
+        <v>551</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>10</v>
       </c>
       <c r="F329">
-        <v>738</v>
+        <v>410</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.25">
@@ -10114,7 +10114,7 @@
         <v>10</v>
       </c>
       <c r="F330">
-        <v>550</v>
+        <v>872</v>
       </c>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.25">
@@ -10134,7 +10134,7 @@
         <v>10</v>
       </c>
       <c r="F331">
-        <v>656</v>
+        <v>383</v>
       </c>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.25">
@@ -10154,7 +10154,7 @@
         <v>10</v>
       </c>
       <c r="F332">
-        <v>920</v>
+        <v>362</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.25">
@@ -10174,7 +10174,7 @@
         <v>10</v>
       </c>
       <c r="F333">
-        <v>224</v>
+        <v>374</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.25">
@@ -10194,7 +10194,7 @@
         <v>10</v>
       </c>
       <c r="F334">
-        <v>838</v>
+        <v>228</v>
       </c>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.25">
@@ -10214,7 +10214,7 @@
         <v>10</v>
       </c>
       <c r="F335">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.25">
@@ -10234,7 +10234,7 @@
         <v>10</v>
       </c>
       <c r="F336">
-        <v>901</v>
+        <v>670</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.25">
@@ -10254,7 +10254,7 @@
         <v>10</v>
       </c>
       <c r="F337">
-        <v>304</v>
+        <v>611</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.25">
@@ -10274,7 +10274,7 @@
         <v>10</v>
       </c>
       <c r="F338">
-        <v>782</v>
+        <v>734</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.25">
@@ -10294,7 +10294,7 @@
         <v>10</v>
       </c>
       <c r="F339">
-        <v>513</v>
+        <v>300</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.25">
@@ -10314,7 +10314,7 @@
         <v>10</v>
       </c>
       <c r="F340">
-        <v>937</v>
+        <v>413</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.25">
@@ -10334,7 +10334,7 @@
         <v>10</v>
       </c>
       <c r="F341">
-        <v>439</v>
+        <v>519</v>
       </c>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.25">
@@ -10354,7 +10354,7 @@
         <v>10</v>
       </c>
       <c r="F342">
-        <v>242</v>
+        <v>260</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.25">
@@ -10374,7 +10374,7 @@
         <v>10</v>
       </c>
       <c r="F343">
-        <v>546</v>
+        <v>922</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.25">
@@ -10394,7 +10394,7 @@
         <v>10</v>
       </c>
       <c r="F344">
-        <v>627</v>
+        <v>747</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.25">
@@ -10414,7 +10414,7 @@
         <v>10</v>
       </c>
       <c r="F345">
-        <v>629</v>
+        <v>832</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.25">
@@ -10434,7 +10434,7 @@
         <v>10</v>
       </c>
       <c r="F346">
-        <v>501</v>
+        <v>652</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.25">
@@ -10454,7 +10454,7 @@
         <v>10</v>
       </c>
       <c r="F347">
-        <v>632</v>
+        <v>414</v>
       </c>
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.25">
@@ -10474,7 +10474,7 @@
         <v>10</v>
       </c>
       <c r="F348">
-        <v>718</v>
+        <v>977</v>
       </c>
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.25">
@@ -10494,7 +10494,7 @@
         <v>10</v>
       </c>
       <c r="F349">
-        <v>754</v>
+        <v>845</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.25">
@@ -10514,7 +10514,7 @@
         <v>10</v>
       </c>
       <c r="F350">
-        <v>653</v>
+        <v>430</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.25">
@@ -10534,7 +10534,7 @@
         <v>10</v>
       </c>
       <c r="F351">
-        <v>894</v>
+        <v>227</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.25">
@@ -10554,7 +10554,7 @@
         <v>10</v>
       </c>
       <c r="F352">
-        <v>526</v>
+        <v>746</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.25">
@@ -10574,7 +10574,7 @@
         <v>10</v>
       </c>
       <c r="F353">
-        <v>861</v>
+        <v>910</v>
       </c>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.25">
@@ -10594,7 +10594,7 @@
         <v>10</v>
       </c>
       <c r="F354">
-        <v>266</v>
+        <v>416</v>
       </c>
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.25">
@@ -10614,7 +10614,7 @@
         <v>10</v>
       </c>
       <c r="F355">
-        <v>227</v>
+        <v>757</v>
       </c>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.25">
@@ -10634,7 +10634,7 @@
         <v>10</v>
       </c>
       <c r="F356">
-        <v>358</v>
+        <v>270</v>
       </c>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.25">
@@ -10654,7 +10654,7 @@
         <v>10</v>
       </c>
       <c r="F357">
-        <v>788</v>
+        <v>586</v>
       </c>
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>10</v>
       </c>
       <c r="F358">
-        <v>657</v>
+        <v>583</v>
       </c>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.25">
@@ -10694,7 +10694,7 @@
         <v>10</v>
       </c>
       <c r="F359">
-        <v>990</v>
+        <v>545</v>
       </c>
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.25">
@@ -10714,7 +10714,7 @@
         <v>10</v>
       </c>
       <c r="F360">
-        <v>996</v>
+        <v>618</v>
       </c>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.25">
@@ -10734,7 +10734,7 @@
         <v>10</v>
       </c>
       <c r="F361">
-        <v>271</v>
+        <v>294</v>
       </c>
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.25">
@@ -10754,7 +10754,7 @@
         <v>10</v>
       </c>
       <c r="F362">
-        <v>737</v>
+        <v>563</v>
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.25">
@@ -10774,7 +10774,7 @@
         <v>10</v>
       </c>
       <c r="F363">
-        <v>918</v>
+        <v>420</v>
       </c>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.25">
@@ -10794,7 +10794,7 @@
         <v>10</v>
       </c>
       <c r="F364">
-        <v>584</v>
+        <v>688</v>
       </c>
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.25">
@@ -10814,7 +10814,7 @@
         <v>10</v>
       </c>
       <c r="F365">
-        <v>562</v>
+        <v>453</v>
       </c>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.25">
@@ -10834,7 +10834,7 @@
         <v>10</v>
       </c>
       <c r="F366">
-        <v>589</v>
+        <v>780</v>
       </c>
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.25">
@@ -10854,7 +10854,7 @@
         <v>10</v>
       </c>
       <c r="F367">
-        <v>312</v>
+        <v>236</v>
       </c>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.25">
@@ -10874,7 +10874,7 @@
         <v>10</v>
       </c>
       <c r="F368">
-        <v>256</v>
+        <v>830</v>
       </c>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.25">
@@ -10894,7 +10894,7 @@
         <v>10</v>
       </c>
       <c r="F369">
-        <v>790</v>
+        <v>648</v>
       </c>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.25">
@@ -10914,7 +10914,7 @@
         <v>10</v>
       </c>
       <c r="F370">
-        <v>854</v>
+        <v>720</v>
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.25">
@@ -10934,7 +10934,7 @@
         <v>10</v>
       </c>
       <c r="F371">
-        <v>851</v>
+        <v>374</v>
       </c>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.25">
@@ -10954,7 +10954,7 @@
         <v>10</v>
       </c>
       <c r="F372">
-        <v>967</v>
+        <v>633</v>
       </c>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.25">
@@ -10974,7 +10974,7 @@
         <v>10</v>
       </c>
       <c r="F373">
-        <v>222</v>
+        <v>252</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.25">
@@ -10994,7 +10994,7 @@
         <v>10</v>
       </c>
       <c r="F374">
-        <v>843</v>
+        <v>922</v>
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.25">
@@ -11014,7 +11014,7 @@
         <v>10</v>
       </c>
       <c r="F375">
-        <v>937</v>
+        <v>605</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.25">
@@ -11034,7 +11034,7 @@
         <v>10</v>
       </c>
       <c r="F376">
-        <v>761</v>
+        <v>473</v>
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.25">
@@ -11054,7 +11054,7 @@
         <v>10</v>
       </c>
       <c r="F377">
-        <v>966</v>
+        <v>415</v>
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.25">
@@ -11074,7 +11074,7 @@
         <v>10</v>
       </c>
       <c r="F378">
-        <v>668</v>
+        <v>251</v>
       </c>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.25">
@@ -11094,7 +11094,7 @@
         <v>10</v>
       </c>
       <c r="F379">
-        <v>577</v>
+        <v>951</v>
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.25">
@@ -11114,7 +11114,7 @@
         <v>10</v>
       </c>
       <c r="F380">
-        <v>497</v>
+        <v>946</v>
       </c>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.25">
@@ -11134,7 +11134,7 @@
         <v>10</v>
       </c>
       <c r="F381">
-        <v>517</v>
+        <v>820</v>
       </c>
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.25">
@@ -11154,7 +11154,7 @@
         <v>10</v>
       </c>
       <c r="F382">
-        <v>249</v>
+        <v>985</v>
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.25">
@@ -11174,7 +11174,7 @@
         <v>10</v>
       </c>
       <c r="F383">
-        <v>868</v>
+        <v>795</v>
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.25">
@@ -11194,7 +11194,7 @@
         <v>10</v>
       </c>
       <c r="F384">
-        <v>397</v>
+        <v>449</v>
       </c>
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.25">
@@ -11214,7 +11214,7 @@
         <v>10</v>
       </c>
       <c r="F385">
-        <v>571</v>
+        <v>452</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.25">
@@ -11234,7 +11234,7 @@
         <v>10</v>
       </c>
       <c r="F386">
-        <v>945</v>
+        <v>624</v>
       </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.25">
@@ -11254,7 +11254,7 @@
         <v>10</v>
       </c>
       <c r="F387">
-        <v>394</v>
+        <v>475</v>
       </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.25">
@@ -11274,7 +11274,7 @@
         <v>10</v>
       </c>
       <c r="F388">
-        <v>219</v>
+        <v>407</v>
       </c>
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.25">
@@ -11294,7 +11294,7 @@
         <v>10</v>
       </c>
       <c r="F389">
-        <v>970</v>
+        <v>609</v>
       </c>
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.25">
@@ -11314,7 +11314,7 @@
         <v>10</v>
       </c>
       <c r="F390">
-        <v>203</v>
+        <v>832</v>
       </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.25">
@@ -11334,7 +11334,7 @@
         <v>10</v>
       </c>
       <c r="F391">
-        <v>449</v>
+        <v>924</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.25">
@@ -11354,7 +11354,7 @@
         <v>10</v>
       </c>
       <c r="F392">
-        <v>518</v>
+        <v>464</v>
       </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.25">
@@ -11374,7 +11374,7 @@
         <v>10</v>
       </c>
       <c r="F393">
-        <v>733</v>
+        <v>538</v>
       </c>
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.25">
@@ -11394,7 +11394,7 @@
         <v>10</v>
       </c>
       <c r="F394">
-        <v>910</v>
+        <v>466</v>
       </c>
     </row>
     <row r="395" spans="1:6" x14ac:dyDescent="0.25">
@@ -11414,7 +11414,7 @@
         <v>10</v>
       </c>
       <c r="F395">
-        <v>913</v>
+        <v>257</v>
       </c>
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.25">
@@ -11434,7 +11434,7 @@
         <v>10</v>
       </c>
       <c r="F396">
-        <v>946</v>
+        <v>652</v>
       </c>
     </row>
     <row r="397" spans="1:6" x14ac:dyDescent="0.25">
@@ -11454,7 +11454,7 @@
         <v>10</v>
       </c>
       <c r="F397">
-        <v>903</v>
+        <v>426</v>
       </c>
     </row>
     <row r="398" spans="1:6" x14ac:dyDescent="0.25">
@@ -11474,7 +11474,7 @@
         <v>10</v>
       </c>
       <c r="F398">
-        <v>571</v>
+        <v>671</v>
       </c>
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.25">
@@ -11494,7 +11494,7 @@
         <v>10</v>
       </c>
       <c r="F399">
-        <v>455</v>
+        <v>414</v>
       </c>
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.25">
@@ -11514,7 +11514,7 @@
         <v>10</v>
       </c>
       <c r="F400">
-        <v>982</v>
+        <v>312</v>
       </c>
     </row>
     <row r="401" spans="1:6" x14ac:dyDescent="0.25">
@@ -11534,7 +11534,7 @@
         <v>10</v>
       </c>
       <c r="F401">
-        <v>500</v>
+        <v>658</v>
       </c>
     </row>
     <row r="402" spans="1:6" x14ac:dyDescent="0.25">
@@ -11554,7 +11554,7 @@
         <v>10</v>
       </c>
       <c r="F402">
-        <v>607</v>
+        <v>340</v>
       </c>
     </row>
     <row r="403" spans="1:6" x14ac:dyDescent="0.25">
@@ -11574,7 +11574,7 @@
         <v>10</v>
       </c>
       <c r="F403">
-        <v>514</v>
+        <v>879</v>
       </c>
     </row>
     <row r="404" spans="1:6" x14ac:dyDescent="0.25">
@@ -11594,7 +11594,7 @@
         <v>10</v>
       </c>
       <c r="F404">
-        <v>543</v>
+        <v>365</v>
       </c>
     </row>
     <row r="405" spans="1:6" x14ac:dyDescent="0.25">
@@ -11614,7 +11614,7 @@
         <v>10</v>
       </c>
       <c r="F405">
-        <v>676</v>
+        <v>909</v>
       </c>
     </row>
     <row r="406" spans="1:6" x14ac:dyDescent="0.25">
@@ -11634,7 +11634,7 @@
         <v>10</v>
       </c>
       <c r="F406">
-        <v>862</v>
+        <v>804</v>
       </c>
     </row>
     <row r="407" spans="1:6" x14ac:dyDescent="0.25">
@@ -11654,7 +11654,7 @@
         <v>10</v>
       </c>
       <c r="F407">
-        <v>689</v>
+        <v>966</v>
       </c>
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.25">
@@ -11674,7 +11674,7 @@
         <v>10</v>
       </c>
       <c r="F408">
-        <v>300</v>
+        <v>962</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.25">
@@ -11694,7 +11694,7 @@
         <v>10</v>
       </c>
       <c r="F409">
-        <v>558</v>
+        <v>254</v>
       </c>
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.25">
@@ -11714,7 +11714,7 @@
         <v>10</v>
       </c>
       <c r="F410">
-        <v>210</v>
+        <v>291</v>
       </c>
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.25">
@@ -11734,7 +11734,7 @@
         <v>10</v>
       </c>
       <c r="F411">
-        <v>757</v>
+        <v>584</v>
       </c>
     </row>
     <row r="412" spans="1:6" x14ac:dyDescent="0.25">
@@ -11754,7 +11754,7 @@
         <v>10</v>
       </c>
       <c r="F412">
-        <v>883</v>
+        <v>460</v>
       </c>
     </row>
     <row r="413" spans="1:6" x14ac:dyDescent="0.25">
@@ -11774,7 +11774,7 @@
         <v>10</v>
       </c>
       <c r="F413">
-        <v>993</v>
+        <v>231</v>
       </c>
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.25">
@@ -11794,7 +11794,7 @@
         <v>10</v>
       </c>
       <c r="F414">
-        <v>569</v>
+        <v>608</v>
       </c>
     </row>
     <row r="415" spans="1:6" x14ac:dyDescent="0.25">
@@ -11814,7 +11814,7 @@
         <v>10</v>
       </c>
       <c r="F415">
-        <v>556</v>
+        <v>421</v>
       </c>
     </row>
     <row r="416" spans="1:6" x14ac:dyDescent="0.25">
@@ -11834,7 +11834,7 @@
         <v>10</v>
       </c>
       <c r="F416">
-        <v>428</v>
+        <v>906</v>
       </c>
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.25">
@@ -11854,7 +11854,7 @@
         <v>10</v>
       </c>
       <c r="F417">
-        <v>588</v>
+        <v>399</v>
       </c>
     </row>
     <row r="418" spans="1:6" x14ac:dyDescent="0.25">
@@ -11874,7 +11874,7 @@
         <v>10</v>
       </c>
       <c r="F418">
-        <v>421</v>
+        <v>896</v>
       </c>
     </row>
     <row r="419" spans="1:6" x14ac:dyDescent="0.25">
@@ -11894,7 +11894,7 @@
         <v>10</v>
       </c>
       <c r="F419">
-        <v>968</v>
+        <v>245</v>
       </c>
     </row>
     <row r="420" spans="1:6" x14ac:dyDescent="0.25">
@@ -11914,7 +11914,7 @@
         <v>10</v>
       </c>
       <c r="F420">
-        <v>623</v>
+        <v>733</v>
       </c>
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.25">
@@ -11934,7 +11934,7 @@
         <v>10</v>
       </c>
       <c r="F421">
-        <v>904</v>
+        <v>917</v>
       </c>
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.25">
@@ -11954,7 +11954,7 @@
         <v>10</v>
       </c>
       <c r="F422">
-        <v>826</v>
+        <v>819</v>
       </c>
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.25">
@@ -11974,7 +11974,7 @@
         <v>10</v>
       </c>
       <c r="F423">
-        <v>425</v>
+        <v>400</v>
       </c>
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.25">
@@ -11994,7 +11994,7 @@
         <v>10</v>
       </c>
       <c r="F424">
-        <v>258</v>
+        <v>812</v>
       </c>
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.25">
@@ -12014,7 +12014,7 @@
         <v>10</v>
       </c>
       <c r="F425">
-        <v>329</v>
+        <v>410</v>
       </c>
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.25">
@@ -12034,7 +12034,7 @@
         <v>10</v>
       </c>
       <c r="F426">
-        <v>280</v>
+        <v>336</v>
       </c>
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.25">
@@ -12054,7 +12054,7 @@
         <v>10</v>
       </c>
       <c r="F427">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.25">
@@ -12074,7 +12074,7 @@
         <v>10</v>
       </c>
       <c r="F428">
-        <v>348</v>
+        <v>467</v>
       </c>
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.25">
@@ -12094,7 +12094,7 @@
         <v>10</v>
       </c>
       <c r="F429">
-        <v>309</v>
+        <v>234</v>
       </c>
     </row>
     <row r="430" spans="1:6" x14ac:dyDescent="0.25">
@@ -12114,7 +12114,7 @@
         <v>10</v>
       </c>
       <c r="F430">
-        <v>829</v>
+        <v>432</v>
       </c>
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.25">
@@ -12134,7 +12134,7 @@
         <v>10</v>
       </c>
       <c r="F431">
-        <v>995</v>
+        <v>872</v>
       </c>
     </row>
     <row r="432" spans="1:6" x14ac:dyDescent="0.25">
@@ -12154,7 +12154,7 @@
         <v>10</v>
       </c>
       <c r="F432">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="433" spans="1:6" x14ac:dyDescent="0.25">
@@ -12174,7 +12174,7 @@
         <v>10</v>
       </c>
       <c r="F433">
-        <v>706</v>
+        <v>898</v>
       </c>
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.25">
@@ -12194,7 +12194,7 @@
         <v>10</v>
       </c>
       <c r="F434">
-        <v>536</v>
+        <v>694</v>
       </c>
     </row>
     <row r="435" spans="1:6" x14ac:dyDescent="0.25">
@@ -12214,7 +12214,7 @@
         <v>10</v>
       </c>
       <c r="F435">
-        <v>767</v>
+        <v>639</v>
       </c>
     </row>
     <row r="436" spans="1:6" x14ac:dyDescent="0.25">
@@ -12234,7 +12234,7 @@
         <v>10</v>
       </c>
       <c r="F436">
-        <v>457</v>
+        <v>521</v>
       </c>
     </row>
     <row r="437" spans="1:6" x14ac:dyDescent="0.25">
@@ -12254,7 +12254,7 @@
         <v>10</v>
       </c>
       <c r="F437">
-        <v>311</v>
+        <v>917</v>
       </c>
     </row>
     <row r="438" spans="1:6" x14ac:dyDescent="0.25">
@@ -12274,7 +12274,7 @@
         <v>10</v>
       </c>
       <c r="F438">
-        <v>969</v>
+        <v>718</v>
       </c>
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.25">
@@ -12294,7 +12294,7 @@
         <v>10</v>
       </c>
       <c r="F439">
-        <v>958</v>
+        <v>654</v>
       </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.25">
@@ -12314,7 +12314,7 @@
         <v>10</v>
       </c>
       <c r="F440">
-        <v>523</v>
+        <v>719</v>
       </c>
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.25">
@@ -12334,7 +12334,7 @@
         <v>10</v>
       </c>
       <c r="F441">
-        <v>223</v>
+        <v>465</v>
       </c>
     </row>
     <row r="442" spans="1:6" x14ac:dyDescent="0.25">
@@ -12354,7 +12354,7 @@
         <v>10</v>
       </c>
       <c r="F442">
-        <v>852</v>
+        <v>937</v>
       </c>
     </row>
     <row r="443" spans="1:6" x14ac:dyDescent="0.25">
@@ -12374,7 +12374,7 @@
         <v>10</v>
       </c>
       <c r="F443">
-        <v>766</v>
+        <v>688</v>
       </c>
     </row>
     <row r="444" spans="1:6" x14ac:dyDescent="0.25">
@@ -12394,7 +12394,7 @@
         <v>10</v>
       </c>
       <c r="F444">
-        <v>219</v>
+        <v>718</v>
       </c>
     </row>
     <row r="445" spans="1:6" x14ac:dyDescent="0.25">
@@ -12414,7 +12414,7 @@
         <v>10</v>
       </c>
       <c r="F445">
-        <v>230</v>
+        <v>562</v>
       </c>
     </row>
     <row r="446" spans="1:6" x14ac:dyDescent="0.25">
@@ -12434,7 +12434,7 @@
         <v>10</v>
       </c>
       <c r="F446">
-        <v>403</v>
+        <v>225</v>
       </c>
     </row>
     <row r="447" spans="1:6" x14ac:dyDescent="0.25">
@@ -12454,7 +12454,7 @@
         <v>10</v>
       </c>
       <c r="F447">
-        <v>893</v>
+        <v>981</v>
       </c>
     </row>
     <row r="448" spans="1:6" x14ac:dyDescent="0.25">
@@ -12474,7 +12474,7 @@
         <v>10</v>
       </c>
       <c r="F448">
-        <v>966</v>
+        <v>758</v>
       </c>
     </row>
     <row r="449" spans="1:6" x14ac:dyDescent="0.25">
@@ -12494,7 +12494,7 @@
         <v>10</v>
       </c>
       <c r="F449">
-        <v>218</v>
+        <v>843</v>
       </c>
     </row>
     <row r="450" spans="1:6" x14ac:dyDescent="0.25">
@@ -12514,7 +12514,7 @@
         <v>10</v>
       </c>
       <c r="F450">
-        <v>481</v>
+        <v>902</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.25">
@@ -12534,7 +12534,7 @@
         <v>10</v>
       </c>
       <c r="F451">
-        <v>529</v>
+        <v>445</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.25">
@@ -12554,7 +12554,7 @@
         <v>10</v>
       </c>
       <c r="F452">
-        <v>868</v>
+        <v>638</v>
       </c>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.25">
@@ -12574,7 +12574,7 @@
         <v>10</v>
       </c>
       <c r="F453">
-        <v>398</v>
+        <v>763</v>
       </c>
     </row>
     <row r="454" spans="1:6" x14ac:dyDescent="0.25">
@@ -12594,7 +12594,7 @@
         <v>10</v>
       </c>
       <c r="F454">
-        <v>220</v>
+        <v>561</v>
       </c>
     </row>
     <row r="455" spans="1:6" x14ac:dyDescent="0.25">
@@ -12614,7 +12614,7 @@
         <v>10</v>
       </c>
       <c r="F455">
-        <v>511</v>
+        <v>989</v>
       </c>
     </row>
     <row r="456" spans="1:6" x14ac:dyDescent="0.25">
@@ -12634,7 +12634,7 @@
         <v>10</v>
       </c>
       <c r="F456">
-        <v>472</v>
+        <v>912</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.25">
@@ -12654,7 +12654,7 @@
         <v>10</v>
       </c>
       <c r="F457">
-        <v>216</v>
+        <v>418</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.25">
@@ -12674,7 +12674,7 @@
         <v>10</v>
       </c>
       <c r="F458">
-        <v>699</v>
+        <v>676</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.25">
@@ -12694,7 +12694,7 @@
         <v>10</v>
       </c>
       <c r="F459">
-        <v>374</v>
+        <v>608</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.25">
@@ -12714,7 +12714,7 @@
         <v>10</v>
       </c>
       <c r="F460">
-        <v>328</v>
+        <v>633</v>
       </c>
     </row>
     <row r="461" spans="1:6" x14ac:dyDescent="0.25">
@@ -12734,7 +12734,7 @@
         <v>10</v>
       </c>
       <c r="F461">
-        <v>531</v>
+        <v>220</v>
       </c>
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.25">
@@ -12754,7 +12754,7 @@
         <v>10</v>
       </c>
       <c r="F462">
-        <v>727</v>
+        <v>288</v>
       </c>
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.25">
@@ -12774,7 +12774,7 @@
         <v>10</v>
       </c>
       <c r="F463">
-        <v>320</v>
+        <v>589</v>
       </c>
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.25">
@@ -12794,7 +12794,7 @@
         <v>10</v>
       </c>
       <c r="F464">
-        <v>421</v>
+        <v>431</v>
       </c>
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.25">
@@ -12814,7 +12814,7 @@
         <v>10</v>
       </c>
       <c r="F465">
-        <v>247</v>
+        <v>309</v>
       </c>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.25">
@@ -12834,7 +12834,7 @@
         <v>10</v>
       </c>
       <c r="F466">
-        <v>626</v>
+        <v>589</v>
       </c>
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.25">
@@ -12854,7 +12854,7 @@
         <v>10</v>
       </c>
       <c r="F467">
-        <v>386</v>
+        <v>637</v>
       </c>
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.25">
@@ -12874,7 +12874,7 @@
         <v>10</v>
       </c>
       <c r="F468">
-        <v>780</v>
+        <v>786</v>
       </c>
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.25">
@@ -12894,7 +12894,7 @@
         <v>10</v>
       </c>
       <c r="F469">
-        <v>576</v>
+        <v>827</v>
       </c>
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.25">
@@ -12914,7 +12914,7 @@
         <v>10</v>
       </c>
       <c r="F470">
-        <v>584</v>
+        <v>510</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.25">
@@ -12934,7 +12934,7 @@
         <v>10</v>
       </c>
       <c r="F471">
-        <v>211</v>
+        <v>743</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.25">
@@ -12954,7 +12954,7 @@
         <v>10</v>
       </c>
       <c r="F472">
-        <v>943</v>
+        <v>666</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.25">
@@ -12974,7 +12974,7 @@
         <v>10</v>
       </c>
       <c r="F473">
-        <v>345</v>
+        <v>723</v>
       </c>
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.25">
@@ -12994,7 +12994,7 @@
         <v>10</v>
       </c>
       <c r="F474">
-        <v>613</v>
+        <v>857</v>
       </c>
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.25">
@@ -13014,7 +13014,7 @@
         <v>10</v>
       </c>
       <c r="F475">
-        <v>697</v>
+        <v>454</v>
       </c>
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.25">
@@ -13034,7 +13034,7 @@
         <v>10</v>
       </c>
       <c r="F476">
-        <v>780</v>
+        <v>879</v>
       </c>
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.25">
@@ -13054,7 +13054,7 @@
         <v>10</v>
       </c>
       <c r="F477">
-        <v>239</v>
+        <v>257</v>
       </c>
     </row>
     <row r="478" spans="1:6" x14ac:dyDescent="0.25">
@@ -13074,7 +13074,7 @@
         <v>10</v>
       </c>
       <c r="F478">
-        <v>951</v>
+        <v>780</v>
       </c>
     </row>
     <row r="479" spans="1:6" x14ac:dyDescent="0.25">
@@ -13094,7 +13094,7 @@
         <v>10</v>
       </c>
       <c r="F479">
-        <v>326</v>
+        <v>726</v>
       </c>
     </row>
     <row r="480" spans="1:6" x14ac:dyDescent="0.25">
@@ -13114,7 +13114,7 @@
         <v>10</v>
       </c>
       <c r="F480">
-        <v>538</v>
+        <v>698</v>
       </c>
     </row>
     <row r="481" spans="1:6" x14ac:dyDescent="0.25">
@@ -13134,7 +13134,7 @@
         <v>10</v>
       </c>
       <c r="F481">
-        <v>833</v>
+        <v>880</v>
       </c>
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.25">
@@ -13154,7 +13154,7 @@
         <v>10</v>
       </c>
       <c r="F482">
-        <v>571</v>
+        <v>913</v>
       </c>
     </row>
     <row r="483" spans="1:6" x14ac:dyDescent="0.25">
@@ -13174,7 +13174,7 @@
         <v>10</v>
       </c>
       <c r="F483">
-        <v>862</v>
+        <v>852</v>
       </c>
     </row>
     <row r="484" spans="1:6" x14ac:dyDescent="0.25">
@@ -13194,7 +13194,7 @@
         <v>10</v>
       </c>
       <c r="F484">
-        <v>323</v>
+        <v>945</v>
       </c>
     </row>
     <row r="485" spans="1:6" x14ac:dyDescent="0.25">
@@ -13214,7 +13214,7 @@
         <v>10</v>
       </c>
       <c r="F485">
-        <v>294</v>
+        <v>270</v>
       </c>
     </row>
     <row r="486" spans="1:6" x14ac:dyDescent="0.25">
@@ -13234,7 +13234,7 @@
         <v>10</v>
       </c>
       <c r="F486">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
     <row r="487" spans="1:6" x14ac:dyDescent="0.25">
@@ -13254,7 +13254,7 @@
         <v>10</v>
       </c>
       <c r="F487">
-        <v>545</v>
+        <v>885</v>
       </c>
     </row>
     <row r="488" spans="1:6" x14ac:dyDescent="0.25">
@@ -13274,7 +13274,7 @@
         <v>10</v>
       </c>
       <c r="F488">
-        <v>974</v>
+        <v>374</v>
       </c>
     </row>
     <row r="489" spans="1:6" x14ac:dyDescent="0.25">
@@ -13294,7 +13294,7 @@
         <v>10</v>
       </c>
       <c r="F489">
-        <v>743</v>
+        <v>782</v>
       </c>
     </row>
     <row r="490" spans="1:6" x14ac:dyDescent="0.25">
@@ -13314,7 +13314,7 @@
         <v>10</v>
       </c>
       <c r="F490">
-        <v>281</v>
+        <v>219</v>
       </c>
     </row>
     <row r="491" spans="1:6" x14ac:dyDescent="0.25">
@@ -13334,7 +13334,7 @@
         <v>10</v>
       </c>
       <c r="F491">
-        <v>886</v>
+        <v>417</v>
       </c>
     </row>
     <row r="492" spans="1:6" x14ac:dyDescent="0.25">
@@ -13354,7 +13354,7 @@
         <v>10</v>
       </c>
       <c r="F492">
-        <v>724</v>
+        <v>586</v>
       </c>
     </row>
     <row r="493" spans="1:6" x14ac:dyDescent="0.25">
@@ -13374,7 +13374,7 @@
         <v>10</v>
       </c>
       <c r="F493">
-        <v>651</v>
+        <v>200</v>
       </c>
     </row>
     <row r="494" spans="1:6" x14ac:dyDescent="0.25">
@@ -13394,7 +13394,7 @@
         <v>10</v>
       </c>
       <c r="F494">
-        <v>725</v>
+        <v>855</v>
       </c>
     </row>
     <row r="495" spans="1:6" x14ac:dyDescent="0.25">
@@ -13414,7 +13414,7 @@
         <v>10</v>
       </c>
       <c r="F495">
-        <v>828</v>
+        <v>745</v>
       </c>
     </row>
     <row r="496" spans="1:6" x14ac:dyDescent="0.25">
@@ -13434,7 +13434,7 @@
         <v>10</v>
       </c>
       <c r="F496">
-        <v>902</v>
+        <v>767</v>
       </c>
     </row>
     <row r="497" spans="1:6" x14ac:dyDescent="0.25">
@@ -13454,7 +13454,7 @@
         <v>10</v>
       </c>
       <c r="F497">
-        <v>592</v>
+        <v>530</v>
       </c>
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.25">
@@ -13474,7 +13474,7 @@
         <v>10</v>
       </c>
       <c r="F498">
-        <v>934</v>
+        <v>553</v>
       </c>
     </row>
     <row r="499" spans="1:6" x14ac:dyDescent="0.25">
@@ -13494,7 +13494,7 @@
         <v>10</v>
       </c>
       <c r="F499">
-        <v>771</v>
+        <v>442</v>
       </c>
     </row>
     <row r="500" spans="1:6" x14ac:dyDescent="0.25">
@@ -13514,7 +13514,7 @@
         <v>10</v>
       </c>
       <c r="F500">
-        <v>780</v>
+        <v>200</v>
       </c>
     </row>
     <row r="501" spans="1:6" x14ac:dyDescent="0.25">
@@ -13534,7 +13534,7 @@
         <v>10</v>
       </c>
       <c r="F501">
-        <v>424</v>
+        <v>757</v>
       </c>
     </row>
     <row r="502" spans="1:6" x14ac:dyDescent="0.25">
@@ -13554,7 +13554,7 @@
         <v>10</v>
       </c>
       <c r="F502">
-        <v>844</v>
+        <v>893</v>
       </c>
     </row>
     <row r="503" spans="1:6" x14ac:dyDescent="0.25">
@@ -13574,7 +13574,7 @@
         <v>10</v>
       </c>
       <c r="F503">
-        <v>702</v>
+        <v>997</v>
       </c>
     </row>
     <row r="504" spans="1:6" x14ac:dyDescent="0.25">
@@ -13594,7 +13594,7 @@
         <v>10</v>
       </c>
       <c r="F504">
-        <v>803</v>
+        <v>426</v>
       </c>
     </row>
     <row r="505" spans="1:6" x14ac:dyDescent="0.25">
@@ -13614,7 +13614,7 @@
         <v>10</v>
       </c>
       <c r="F505">
-        <v>497</v>
+        <v>993</v>
       </c>
     </row>
     <row r="506" spans="1:6" x14ac:dyDescent="0.25">
@@ -13634,7 +13634,7 @@
         <v>10</v>
       </c>
       <c r="F506">
-        <v>911</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>